<commit_message>
Publish updates example dataset
</commit_message>
<xml_diff>
--- a/docs/sample_data/athabasca_rbt/stressor_response_demo.xlsx
+++ b/docs/sample_data/athabasca_rbt/stressor_response_demo.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25330"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF73DDF8-EF8C-410A-AB28-B28527926417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334F6A88-B3A3-4C41-97BC-9029FB7D9C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="525" windowWidth="29040" windowHeight="15720" firstSheet="8" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="2" r:id="rId1"/>
@@ -24,8 +24,7 @@
     <sheet name="Selenium" sheetId="20" r:id="rId14"/>
     <sheet name="WD" sheetId="21" r:id="rId15"/>
     <sheet name="Habitat_loss" sheetId="22" r:id="rId16"/>
-    <sheet name="Spring_flow_alevin" sheetId="24" r:id="rId17"/>
-    <sheet name="Spring_flow_sub" sheetId="25" r:id="rId18"/>
+    <sheet name="Spring_flow_sub" sheetId="25" r:id="rId17"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -261,7 +260,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="45">
   <si>
     <t>Stressors</t>
   </si>
@@ -380,13 +379,7 @@
     <t>capacity</t>
   </si>
   <si>
-    <t>Spring_flow_alevin</t>
-  </si>
-  <si>
     <t>Spring_flow</t>
-  </si>
-  <si>
-    <t>alevin</t>
   </si>
   <si>
     <t>Spring_flow_sub</t>
@@ -402,12 +395,6 @@
   </si>
   <si>
     <t>All</t>
-  </si>
-  <si>
-    <t>Population Model</t>
-  </si>
-  <si>
-    <t>Joe Model</t>
   </si>
 </sst>
 </file>
@@ -491,7 +478,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="6"/>
@@ -505,14 +492,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -14367,7 +14350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.44140625" style="2" customWidth="1"/>
@@ -14400,536 +14383,505 @@
       <c r="F1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="I1" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>45</v>
+      <c r="I1" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="2" t="s">
         <v>34</v>
       </c>
       <c r="I2" s="5"/>
       <c r="J2" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="K2" s="6"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="2" t="s">
         <v>34</v>
       </c>
       <c r="I3" s="5"/>
       <c r="J3" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="K3" s="6"/>
     </row>
     <row r="4" spans="1:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H4" s="8"/>
+      <c r="H4" s="2"/>
       <c r="I4" s="5"/>
       <c r="J4" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K4" s="6"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H5" s="8"/>
+      <c r="H5" s="2"/>
       <c r="I5" s="5"/>
       <c r="J5" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K5" s="6"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H6" s="8"/>
+      <c r="H6" s="2"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K6" s="6"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H7" s="8"/>
-      <c r="I7" s="7"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="6"/>
       <c r="J7" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K7" s="6"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H8" s="8"/>
-      <c r="I8" s="7"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="6"/>
       <c r="J8" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K8" s="6"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H9" s="8"/>
-      <c r="I9" s="7"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="6"/>
       <c r="J9" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K9" s="6"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H10" s="8"/>
-      <c r="I10" s="7"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="6"/>
       <c r="J10" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K10" s="6"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H11" s="8"/>
-      <c r="I11" s="7"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="6"/>
       <c r="J11" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K11" s="6"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H12" s="8"/>
-      <c r="I12" s="7"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="6"/>
       <c r="J12" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K12" s="6"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H13" s="8"/>
-      <c r="I13" s="7"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="6"/>
       <c r="J13" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K13" s="6"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H14" s="8"/>
-      <c r="I14" s="7"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="6"/>
       <c r="J14" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K14" s="6"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H15" s="8"/>
-      <c r="I15" s="7"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="6"/>
       <c r="J15" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="K15" s="6"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G16" s="8" t="s">
+      <c r="G16" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H16" s="8" t="s">
+      <c r="H16" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I16" s="7"/>
+      <c r="I16" s="6"/>
       <c r="J16" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="K16" s="6"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H17" s="8" t="s">
+      <c r="H17" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="I17" s="7"/>
+      <c r="I17" s="6"/>
       <c r="J17" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="K17" s="6"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A18" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="I18" s="7"/>
-      <c r="J18" s="5" t="s">
-        <v>47</v>
-      </c>
+      <c r="I18" s="6"/>
+      <c r="J18" s="6"/>
       <c r="K18" s="6"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="I19" s="7"/>
-      <c r="J19" s="7"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
       <c r="K19" s="6"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="I20" s="6"/>
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16236,326 +16188,6 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57FA864D-7D9A-4124-BBDE-66EA81ABD765}">
-  <dimension ref="A1:E18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2">
-        <v>10</v>
-      </c>
-      <c r="C2">
-        <v>20</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>50</v>
-      </c>
-      <c r="B3">
-        <v>40</v>
-      </c>
-      <c r="C3">
-        <v>20</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>100</v>
-      </c>
-      <c r="B4">
-        <v>60</v>
-      </c>
-      <c r="C4">
-        <v>20</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>150</v>
-      </c>
-      <c r="B5">
-        <v>75</v>
-      </c>
-      <c r="C5">
-        <v>20</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>200</v>
-      </c>
-      <c r="B6">
-        <v>90</v>
-      </c>
-      <c r="C6">
-        <v>20</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>250</v>
-      </c>
-      <c r="B7">
-        <v>100</v>
-      </c>
-      <c r="C7">
-        <v>20</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>300</v>
-      </c>
-      <c r="B8">
-        <v>100</v>
-      </c>
-      <c r="C8">
-        <v>20</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-      <c r="E8">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>350</v>
-      </c>
-      <c r="B9">
-        <v>100</v>
-      </c>
-      <c r="C9">
-        <v>20</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>400</v>
-      </c>
-      <c r="B10">
-        <v>100</v>
-      </c>
-      <c r="C10">
-        <v>20</v>
-      </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>450</v>
-      </c>
-      <c r="B11">
-        <v>100</v>
-      </c>
-      <c r="C11">
-        <v>20</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>500</v>
-      </c>
-      <c r="B12">
-        <v>100</v>
-      </c>
-      <c r="C12">
-        <v>20</v>
-      </c>
-      <c r="D12">
-        <v>0</v>
-      </c>
-      <c r="E12">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>550</v>
-      </c>
-      <c r="B13">
-        <v>100</v>
-      </c>
-      <c r="C13">
-        <v>20</v>
-      </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
-      <c r="E13">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>600</v>
-      </c>
-      <c r="B14">
-        <v>90</v>
-      </c>
-      <c r="C14">
-        <v>20</v>
-      </c>
-      <c r="D14">
-        <v>0</v>
-      </c>
-      <c r="E14">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>650</v>
-      </c>
-      <c r="B15">
-        <v>75</v>
-      </c>
-      <c r="C15">
-        <v>20</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
-      <c r="E15">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>700</v>
-      </c>
-      <c r="B16">
-        <v>60</v>
-      </c>
-      <c r="C16">
-        <v>20</v>
-      </c>
-      <c r="D16">
-        <v>0</v>
-      </c>
-      <c r="E16">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>750</v>
-      </c>
-      <c r="B17">
-        <v>40</v>
-      </c>
-      <c r="C17">
-        <v>20</v>
-      </c>
-      <c r="D17">
-        <v>0</v>
-      </c>
-      <c r="E17">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>800</v>
-      </c>
-      <c r="B18">
-        <v>10</v>
-      </c>
-      <c r="C18">
-        <v>20</v>
-      </c>
-      <c r="D18">
-        <v>0</v>
-      </c>
-      <c r="E18">
-        <v>100</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A82EBC21-D1BB-4053-A20F-EBCCD4B5FB3D}">
   <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -16566,7 +16198,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>6</v>

</xml_diff>